<commit_message>
added reserve ref and jury
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/emptyProtocol/EmptyWithDeclaration-A4.xlsx
+++ b/owlcms/src/main/resources/templates/emptyProtocol/EmptyWithDeclaration-A4.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\emptyProtocol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\emptyProtocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D01008A-98A3-436F-A5BF-BA3EACA030BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7E6632-5A04-43EC-B5E2-D5E1C9D01485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="2805" windowWidth="21600" windowHeight="11295"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Starting Weights" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_1Excel_BuiltIn_Criteria_1_1">'Starting Weights'!#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Starting Weights'!$A$9:$X$9</definedName>
     <definedName name="AFF.">'Starting Weights'!#REF!</definedName>
     <definedName name="Affiliation">'Starting Weights'!#REF!</definedName>
@@ -30,7 +31,6 @@
     <definedName name="dernier">'Starting Weights'!#REF!</definedName>
     <definedName name="essais">'Starting Weights'!#REF!</definedName>
     <definedName name="essaisArr">'Starting Weights'!#REF!</definedName>
-    <definedName name="_1Excel_BuiltIn_Criteria_1_1">'Starting Weights'!#REF!</definedName>
     <definedName name="GroupeCourant">'Starting Weights'!$E$6</definedName>
     <definedName name="Groupes">#REF!</definedName>
     <definedName name="GroupFilter">'Starting Weights'!#REF!</definedName>
@@ -55,21 +55,12 @@
     <definedName name="TAS">'Starting Weights'!#REF!</definedName>
     <definedName name="tirage">'Starting Weights'!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="125725" fullCalcOnLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="125725" iterate="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
   <si>
     <t>&lt;/jx:forEach&gt;</t>
   </si>
@@ -98,21 +89,6 @@
     <t>${competition.competitionOrganizer}</t>
   </si>
   <si>
-    <t>${session.announcer}</t>
-  </si>
-  <si>
-    <t>${session.referee1}</t>
-  </si>
-  <si>
-    <t>${session.referee2}</t>
-  </si>
-  <si>
-    <t>${session.timeKeeper}</t>
-  </si>
-  <si>
-    <t>${session.referee3}</t>
-  </si>
-  <si>
     <t>${l.membership}</t>
   </si>
   <si>
@@ -149,9 +125,6 @@
     <t>&lt;jx:forEach items="${athletes}" var="l" varStatus="lifterLoop"&gt;</t>
   </si>
   <si>
-    <t>${session.jury1} ${session.jury2} ${session.jury3} ${session.jury4} ${session.jury5}</t>
-  </si>
-  <si>
     <t>${l.yearOfBirth}</t>
   </si>
   <si>
@@ -248,21 +221,51 @@
     <t>${competition.localizedCompetitionDate}</t>
   </si>
   <si>
-    <t>${session.marshall} ${session.marshal2}</t>
-  </si>
-  <si>
-    <t>${session.technicalController} ${session.technicalController2}</t>
+    <t>${session.announcerAsTO} ${session.announcerAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.marshallAsTO} ${session.marshallAsTO.federationId} ${session.marshal2AsTO} ${session.marshal2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.timeKeeperAsTO} ${session.timeKeeperAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO} ${session.technicalControllerAsTO.federationId} ${session.technicalController2AsTO} ${session.technicalController2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("Reserve")}</t>
+  </si>
+  <si>
+    <t>${session.referee1AsTO} ${session.referee1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee2AsTO} ${session.referee2AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.referee3AsTO} ${session.referee3AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO} ${session.reserveAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("JuryPresident")}</t>
+  </si>
+  <si>
+    <t>${session.jury1AsTO} ${session.jury1AsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO} ${session.jury2AsTO.federationId} ${session.jury3AsTO} ${session.jury3AsTO.federationId} ${session.jury4AsTO} ${session.jury4AsTO.federationId} ${session.jury5AsTO} ${session.jury5AsTO.federationId} ${session.reserveJuryAsTO != null ? "("+t.get("Reserve")+") "+session.reserveJuryAsTO+" "+session.reserveJuryAsTO.federationId : ""}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="181" formatCode="0.0;;"/>
-    <numFmt numFmtId="183" formatCode="0;\(0\);\-"/>
-    <numFmt numFmtId="184" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
-    <numFmt numFmtId="185" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="0.0;;"/>
+    <numFmt numFmtId="165" formatCode="0;\(0\);\-"/>
+    <numFmt numFmtId="166" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
   </numFmts>
   <fonts count="23" x14ac:knownFonts="1">
     <font>
@@ -567,107 +570,88 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="183" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -677,39 +661,35 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="183" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -727,9 +707,6 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -756,9 +733,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -794,33 +768,40 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="181" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -829,54 +810,47 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
-    <cellStyle name="Emphase 1" xfId="1"/>
-    <cellStyle name="Emphase 2" xfId="2"/>
-    <cellStyle name="Emphase 3" xfId="3"/>
+    <cellStyle name="Emphase 1" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Emphase 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Emphase 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Hyperlink" xfId="4" builtinId="8"/>
-    <cellStyle name="Lien hypertexte 2" xfId="5"/>
+    <cellStyle name="Lien hypertexte 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="6"/>
-    <cellStyle name="Normal 3" xfId="7"/>
-    <cellStyle name="Titre 1" xfId="8"/>
-    <cellStyle name="Titre 1 1" xfId="9"/>
-    <cellStyle name="Titre 1 1 1" xfId="10"/>
-    <cellStyle name="Titre de la feuille" xfId="11"/>
+    <cellStyle name="Normal 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Titre 1" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Titre 1 1" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Titre 1 1 1" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Titre de la feuille" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1306,11 +1280,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X116"/>
+  <dimension ref="A1:Y116"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
@@ -1318,245 +1292,237 @@
     <col min="3" max="3" width="5.7109375" customWidth="1"/>
     <col min="4" max="4" width="36.140625" customWidth="1"/>
     <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="14.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.7109375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="6.85546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="6.85546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="6.5703125" style="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="1" customWidth="1"/>
     <col min="12" max="13" width="7.7109375" style="1" customWidth="1"/>
     <col min="14" max="14" width="7.7109375" customWidth="1"/>
-    <col min="15" max="15" width="7" style="4" customWidth="1"/>
+    <col min="15" max="15" width="7" style="3" customWidth="1"/>
     <col min="16" max="16" width="9.140625" style="1" customWidth="1"/>
     <col min="17" max="18" width="7.7109375" style="1" customWidth="1"/>
     <col min="19" max="19" width="7.7109375" customWidth="1"/>
-    <col min="20" max="20" width="6.85546875" style="2" customWidth="1"/>
-    <col min="21" max="21" width="7.7109375" style="2" customWidth="1"/>
+    <col min="20" max="20" width="6.85546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="7.7109375" style="1" customWidth="1"/>
     <col min="22" max="22" width="7" style="1" customWidth="1"/>
     <col min="23" max="23" width="6.28515625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="11.42578125" style="5" customWidth="1"/>
-    <col min="25" max="25" width="11.42578125" customWidth="1"/>
+    <col min="24" max="25" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
+    <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="50"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="41"/>
       <c r="H1" s="1"/>
-      <c r="J1" s="64" t="s">
-        <v>43</v>
-      </c>
-      <c r="K1" s="100" t="s">
+      <c r="J1" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="100"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
-      <c r="O1" s="100"/>
-      <c r="P1" s="100"/>
-      <c r="Q1" s="100"/>
-      <c r="R1" s="100"/>
-      <c r="S1" s="100"/>
-      <c r="T1" s="100"/>
-      <c r="U1" s="100"/>
-      <c r="V1" s="100"/>
-      <c r="X1"/>
-    </row>
-    <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="67" t="s">
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="81"/>
+      <c r="T1" s="81"/>
+      <c r="U1" s="81"/>
+      <c r="V1" s="81"/>
+    </row>
+    <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="69"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="58"/>
       <c r="F2"/>
       <c r="H2" s="1"/>
-      <c r="J2" s="64" t="s">
-        <v>44</v>
-      </c>
-      <c r="K2" s="70" t="s">
+      <c r="J2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="86"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="64" t="s">
-        <v>45</v>
-      </c>
-      <c r="S2" s="32" t="s">
+      <c r="L2" s="72"/>
+      <c r="M2" s="60"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="61"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" t="s">
         <v>7</v>
       </c>
-      <c r="T2" s="87"/>
-      <c r="U2" s="87"/>
-      <c r="X2"/>
-    </row>
-    <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="73" t="s">
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+    </row>
+    <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="74"/>
+      <c r="B3" s="63"/>
       <c r="F3"/>
       <c r="H3" s="1"/>
-      <c r="J3" s="64" t="s">
-        <v>46</v>
-      </c>
-      <c r="K3" s="89" t="s">
-        <v>58</v>
-      </c>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="89"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="37"/>
-      <c r="R3" s="64" t="s">
-        <v>47</v>
-      </c>
-      <c r="S3" s="75" t="s">
+      <c r="J3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" s="83" t="s">
+        <v>52</v>
+      </c>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="T3" s="76"/>
-      <c r="U3" s="76"/>
-      <c r="V3" s="77"/>
-      <c r="X3"/>
-    </row>
-    <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="73" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="78"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="66"/>
+    </row>
+    <row r="4" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="62"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
       <c r="F4"/>
       <c r="H4" s="1"/>
-      <c r="J4" s="64" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" s="80" t="s">
+      <c r="J4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>6</v>
       </c>
       <c r="L4"/>
-      <c r="M4" s="81"/>
+      <c r="M4" s="3"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="Q4"/>
-      <c r="R4" s="64"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="1"/>
-      <c r="U4" s="1"/>
-      <c r="X4"/>
-    </row>
-    <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:24" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="94" t="s">
+      <c r="R4" s="7"/>
+      <c r="S4" s="69"/>
+    </row>
+    <row r="5" spans="1:25" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="6"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="88" t="s">
+        <v>43</v>
+      </c>
+      <c r="K6" s="88"/>
+      <c r="L6" s="88"/>
+      <c r="M6" s="88"/>
+      <c r="N6" s="88"/>
+      <c r="O6" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="P6" s="89"/>
+      <c r="Q6" s="89"/>
+      <c r="R6" s="89"/>
+      <c r="S6" s="89"/>
+      <c r="T6" s="84" t="s">
+        <v>47</v>
+      </c>
+      <c r="U6" s="84" t="s">
+        <v>46</v>
+      </c>
+      <c r="V6" s="86" t="s">
+        <v>48</v>
+      </c>
+      <c r="W6" s="9"/>
+    </row>
+    <row r="7" spans="1:25" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="71" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="95"/>
-      <c r="L6" s="95"/>
-      <c r="M6" s="95"/>
-      <c r="N6" s="95"/>
-      <c r="O6" s="96" t="s">
+      <c r="J7" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="P6" s="97"/>
-      <c r="Q6" s="97"/>
-      <c r="R6" s="97"/>
-      <c r="S6" s="97"/>
-      <c r="T6" s="90" t="s">
-        <v>53</v>
-      </c>
-      <c r="U6" s="90" t="s">
-        <v>52</v>
-      </c>
-      <c r="V6" s="92" t="s">
-        <v>54</v>
-      </c>
-      <c r="W6" s="14"/>
-    </row>
-    <row r="7" spans="1:24" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="85" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="83" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="K7" s="19">
+      <c r="K7" s="13">
         <v>1</v>
       </c>
-      <c r="L7" s="19">
+      <c r="L7" s="13">
         <v>2</v>
       </c>
-      <c r="M7" s="19">
+      <c r="M7" s="13">
         <v>3</v>
       </c>
-      <c r="N7" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="O7" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="P7" s="19">
+      <c r="N7" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="O7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="P7" s="13">
         <v>1</v>
       </c>
-      <c r="Q7" s="19">
+      <c r="Q7" s="13">
         <v>2</v>
       </c>
-      <c r="R7" s="19">
+      <c r="R7" s="13">
         <v>3</v>
       </c>
-      <c r="S7" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="T7" s="91"/>
-      <c r="U7" s="91"/>
-      <c r="V7" s="93"/>
-      <c r="W7" s="23"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="S7" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="T7" s="85"/>
+      <c r="U7" s="85"/>
+      <c r="V7" s="87"/>
+      <c r="W7" s="17"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F8"/>
       <c r="G8"/>
@@ -1574,60 +1540,59 @@
       <c r="U8"/>
       <c r="V8"/>
       <c r="W8"/>
-      <c r="X8"/>
-    </row>
-    <row r="9" spans="1:24" s="27" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="24" t="s">
+    </row>
+    <row r="9" spans="1:25" s="21" customFormat="1" ht="21.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="J9" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="42"/>
-      <c r="L9" s="42"/>
-      <c r="M9" s="42"/>
-      <c r="N9" s="44"/>
-      <c r="O9" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="P9" s="42"/>
-      <c r="Q9" s="42"/>
-      <c r="R9" s="42"/>
-      <c r="S9" s="44"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="46"/>
-      <c r="V9" s="47"/>
-      <c r="W9" s="26"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="P9" s="34"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="34"/>
+      <c r="S9" s="36"/>
+      <c r="T9" s="37"/>
+      <c r="U9" s="38"/>
+      <c r="V9" s="38"/>
+      <c r="W9" s="20"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
-      <c r="F10" s="32"/>
+      <c r="F10"/>
       <c r="G10"/>
       <c r="H10"/>
       <c r="I10"/>
@@ -1639,515 +1604,544 @@
       <c r="P10"/>
       <c r="Q10"/>
       <c r="R10"/>
-      <c r="S10" s="32"/>
       <c r="T10"/>
       <c r="U10"/>
       <c r="V10"/>
       <c r="W10"/>
-      <c r="X10"/>
-    </row>
-    <row r="11" spans="1:24" s="29" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="48"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="98" t="s">
-        <v>35</v>
-      </c>
-      <c r="G11" s="49"/>
-      <c r="H11" s="50"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="98" t="s">
-        <v>36</v>
-      </c>
-      <c r="K11" s="98"/>
-      <c r="L11" s="48"/>
-      <c r="N11" s="51"/>
-      <c r="P11" s="48"/>
-      <c r="Q11" s="99" t="s">
-        <v>37</v>
-      </c>
-      <c r="R11" s="99"/>
-      <c r="S11" s="52"/>
-      <c r="T11" s="48"/>
-      <c r="U11" s="53"/>
-      <c r="V11" s="48"/>
-      <c r="W11" s="48"/>
-    </row>
-    <row r="12" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:25" s="23" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="79" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="40"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="79" t="s">
+        <v>30</v>
+      </c>
+      <c r="K11" s="79"/>
+      <c r="L11" s="39"/>
+      <c r="N11" s="42"/>
+      <c r="P11" s="39"/>
+      <c r="Q11" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" s="80"/>
+      <c r="S11" s="43"/>
+      <c r="T11" s="39"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="39"/>
+      <c r="W11" s="90"/>
+      <c r="X11" s="91"/>
+      <c r="Y11" s="91"/>
+    </row>
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="54" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="55"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="98"/>
-      <c r="K12" s="98"/>
-      <c r="L12" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="M12" s="55"/>
-      <c r="N12" s="55"/>
-      <c r="O12" s="55"/>
-      <c r="P12" s="56"/>
-      <c r="Q12" s="99"/>
-      <c r="R12" s="99"/>
-      <c r="S12" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="T12" s="56"/>
-      <c r="U12" s="55"/>
-      <c r="V12" s="55"/>
-      <c r="W12"/>
-      <c r="X12"/>
-    </row>
-    <row r="13" spans="1:24" s="30" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="57"/>
-      <c r="B13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="59"/>
-      <c r="I13" s="57"/>
-      <c r="K13" s="60"/>
-      <c r="L13" s="59"/>
-      <c r="M13" s="59"/>
-      <c r="N13" s="59"/>
-      <c r="O13" s="59"/>
-      <c r="P13" s="59"/>
-      <c r="Q13" s="57"/>
-      <c r="S13" s="59"/>
-      <c r="T13" s="59"/>
-      <c r="U13" s="59"/>
-    </row>
-    <row r="14" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="45"/>
+      <c r="E12" s="79"/>
+      <c r="F12" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="79"/>
+      <c r="K12" s="79"/>
+      <c r="L12" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="M12" s="45"/>
+      <c r="N12" s="45"/>
+      <c r="O12" s="45"/>
+      <c r="P12" s="46"/>
+      <c r="Q12" s="80"/>
+      <c r="R12" s="80"/>
+      <c r="S12" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="T12" s="46"/>
+      <c r="U12" s="45"/>
+      <c r="V12" s="73"/>
+      <c r="W12" s="92"/>
+      <c r="X12" s="94"/>
+      <c r="Y12" s="92"/>
+    </row>
+    <row r="13" spans="1:25" s="24" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="47"/>
+      <c r="B13" s="48"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="49"/>
+      <c r="I13" s="47"/>
+      <c r="K13" s="50"/>
+      <c r="L13" s="49"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="49"/>
+      <c r="O13" s="49"/>
+      <c r="P13" s="49"/>
+      <c r="Q13" s="47"/>
+      <c r="S13" s="49"/>
+      <c r="T13" s="49"/>
+      <c r="U13" s="49"/>
+      <c r="V13" s="74"/>
+      <c r="W13" s="93"/>
+      <c r="X13" s="93"/>
+      <c r="Y13" s="93"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="62"/>
+      <c r="B14" s="52"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="48"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="39"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="88" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="88"/>
+      <c r="J14" s="82" t="s">
+        <v>33</v>
+      </c>
+      <c r="K14" s="82"/>
       <c r="M14"/>
       <c r="N14" s="1"/>
-      <c r="O14" s="53"/>
+      <c r="O14" s="22"/>
+      <c r="Q14" s="82" t="s">
+        <v>57</v>
+      </c>
+      <c r="R14" s="82"/>
+      <c r="S14" s="1"/>
       <c r="T14"/>
-      <c r="U14"/>
-      <c r="V14"/>
-      <c r="W14"/>
-      <c r="X14"/>
-    </row>
-    <row r="15" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V14" s="22"/>
+      <c r="W14" s="94"/>
+      <c r="X14" s="92"/>
+      <c r="Y14" s="92"/>
+    </row>
+    <row r="15" spans="1:25" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="54" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="33" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="55"/>
-      <c r="E15" s="54" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15" s="33" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="88"/>
-      <c r="K15" s="88"/>
-      <c r="L15" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="M15" s="56"/>
-      <c r="N15" s="55"/>
-      <c r="O15" s="55"/>
-      <c r="P15" s="55"/>
-      <c r="T15"/>
-      <c r="U15"/>
-      <c r="V15"/>
-      <c r="W15"/>
-      <c r="X15"/>
-    </row>
-    <row r="16" spans="1:24" s="30" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="57"/>
-      <c r="B16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="59"/>
-      <c r="I16" s="57"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="59"/>
-      <c r="M16" s="59"/>
-      <c r="N16" s="59"/>
-      <c r="O16" s="59"/>
-      <c r="P16" s="59"/>
-      <c r="Q16" s="57"/>
-    </row>
-    <row r="17" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="45"/>
+      <c r="E15" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="82"/>
+      <c r="K15" s="82"/>
+      <c r="L15" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="M15" s="46"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="82"/>
+      <c r="R15" s="82"/>
+      <c r="S15" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="T15" s="46"/>
+      <c r="U15" s="45"/>
+      <c r="V15" s="45"/>
+      <c r="W15" s="94"/>
+      <c r="X15" s="92"/>
+      <c r="Y15" s="92"/>
+    </row>
+    <row r="16" spans="1:25" s="24" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="47"/>
+      <c r="B16" s="48"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="49"/>
+      <c r="I16" s="47"/>
+      <c r="K16" s="50"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="47"/>
+      <c r="V16" s="74"/>
+      <c r="W16" s="93"/>
+      <c r="X16" s="93"/>
+      <c r="Y16" s="93"/>
+    </row>
+    <row r="17" spans="1:25" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="62"/>
+      <c r="B17" s="52"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="63"/>
-      <c r="F17" s="48"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="39"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17"/>
-      <c r="K17" s="64"/>
+      <c r="K17" s="7"/>
       <c r="M17"/>
       <c r="N17" s="1"/>
-      <c r="O17" s="53"/>
+      <c r="O17" s="22"/>
       <c r="T17"/>
       <c r="U17"/>
-      <c r="V17"/>
-      <c r="W17"/>
-      <c r="X17"/>
-    </row>
-    <row r="18" spans="1:24" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V17" s="75"/>
+      <c r="W17" s="92"/>
+      <c r="X17" s="92"/>
+      <c r="Y17" s="92"/>
+    </row>
+    <row r="18" spans="1:25" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="54" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" s="33" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="55"/>
-      <c r="N18" s="55"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="55"/>
-      <c r="T18"/>
-      <c r="U18"/>
-      <c r="V18"/>
-      <c r="W18"/>
-      <c r="X18"/>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E19" s="2"/>
-      <c r="U19" s="28"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E20" s="2"/>
-      <c r="U20" s="28"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E21" s="2"/>
-      <c r="U21" s="28"/>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="D22" s="31"/>
-      <c r="E22" s="2"/>
-      <c r="U22" s="28"/>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E23" s="2"/>
-      <c r="U23" s="28"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E24" s="2"/>
-      <c r="U24" s="28"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E31" s="2"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E32" s="2"/>
+      <c r="B18" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="45"/>
+      <c r="E18" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="45"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="45"/>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="76"/>
+      <c r="R18" s="76"/>
+      <c r="S18" s="77"/>
+      <c r="T18" s="77"/>
+      <c r="U18" s="77"/>
+      <c r="V18" s="78"/>
+      <c r="W18" s="92"/>
+      <c r="X18" s="92"/>
+      <c r="Y18" s="92"/>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E19" s="1"/>
+      <c r="U19" s="22"/>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E20" s="1"/>
+      <c r="U20" s="22"/>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E21" s="1"/>
+      <c r="U21" s="22"/>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="D22" s="25"/>
+      <c r="E22" s="1"/>
+      <c r="U22" s="22"/>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E23" s="1"/>
+      <c r="U23" s="22"/>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E24" s="1"/>
+      <c r="U24" s="22"/>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="E32" s="1"/>
     </row>
     <row r="33" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E33" s="2"/>
+      <c r="E33" s="1"/>
     </row>
     <row r="34" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E34" s="2"/>
+      <c r="E34" s="1"/>
     </row>
     <row r="35" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E35" s="2"/>
+      <c r="E35" s="1"/>
     </row>
     <row r="36" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E36" s="2"/>
+      <c r="E36" s="1"/>
     </row>
     <row r="37" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E37" s="2"/>
+      <c r="E37" s="1"/>
     </row>
     <row r="38" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E38" s="2"/>
+      <c r="E38" s="1"/>
     </row>
     <row r="39" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E39" s="2"/>
+      <c r="E39" s="1"/>
     </row>
     <row r="40" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E40" s="2"/>
+      <c r="E40" s="1"/>
     </row>
     <row r="41" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E41" s="2"/>
+      <c r="E41" s="1"/>
     </row>
     <row r="42" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E42" s="2"/>
+      <c r="E42" s="1"/>
     </row>
     <row r="43" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E43" s="2"/>
+      <c r="E43" s="1"/>
     </row>
     <row r="44" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E44" s="2"/>
+      <c r="E44" s="1"/>
     </row>
     <row r="45" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E45" s="2"/>
+      <c r="E45" s="1"/>
     </row>
     <row r="46" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E46" s="2"/>
+      <c r="E46" s="1"/>
     </row>
     <row r="47" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E47" s="2"/>
+      <c r="E47" s="1"/>
     </row>
     <row r="48" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E48" s="2"/>
+      <c r="E48" s="1"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="2"/>
+      <c r="E49" s="1"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="2"/>
+      <c r="E50" s="1"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="2"/>
+      <c r="E51" s="1"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="2"/>
+      <c r="E52" s="1"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="2"/>
+      <c r="E53" s="1"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="2"/>
+      <c r="E54" s="1"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="2"/>
+      <c r="E55" s="1"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="2"/>
+      <c r="E56" s="1"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="2"/>
+      <c r="E57" s="1"/>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E58" s="2"/>
+      <c r="E58" s="1"/>
     </row>
     <row r="59" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E59" s="2"/>
+      <c r="E59" s="1"/>
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E60" s="2"/>
+      <c r="E60" s="1"/>
     </row>
     <row r="61" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E61" s="2"/>
+      <c r="E61" s="1"/>
     </row>
     <row r="62" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E62" s="2"/>
+      <c r="E62" s="1"/>
     </row>
     <row r="63" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E63" s="2"/>
+      <c r="E63" s="1"/>
     </row>
     <row r="64" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E64" s="2"/>
+      <c r="E64" s="1"/>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E65" s="2"/>
+      <c r="E65" s="1"/>
     </row>
     <row r="66" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E66" s="2"/>
+      <c r="E66" s="1"/>
     </row>
     <row r="67" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E67" s="2"/>
+      <c r="E67" s="1"/>
     </row>
     <row r="68" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E68" s="2"/>
+      <c r="E68" s="1"/>
     </row>
     <row r="69" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E69" s="2"/>
+      <c r="E69" s="1"/>
     </row>
     <row r="70" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E70" s="2"/>
+      <c r="E70" s="1"/>
     </row>
     <row r="71" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E71" s="2"/>
+      <c r="E71" s="1"/>
     </row>
     <row r="72" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E72" s="2"/>
+      <c r="E72" s="1"/>
     </row>
     <row r="73" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E73" s="2"/>
+      <c r="E73" s="1"/>
     </row>
     <row r="74" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E74" s="2"/>
+      <c r="E74" s="1"/>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E75" s="2"/>
+      <c r="E75" s="1"/>
     </row>
     <row r="76" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E76" s="2"/>
+      <c r="E76" s="1"/>
     </row>
     <row r="77" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E77" s="2"/>
+      <c r="E77" s="1"/>
     </row>
     <row r="78" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E78" s="2"/>
+      <c r="E78" s="1"/>
     </row>
     <row r="79" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E79" s="2"/>
+      <c r="E79" s="1"/>
     </row>
     <row r="80" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E80" s="2"/>
+      <c r="E80" s="1"/>
     </row>
     <row r="81" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E81" s="2"/>
+      <c r="E81" s="1"/>
     </row>
     <row r="82" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E82" s="2"/>
+      <c r="E82" s="1"/>
     </row>
     <row r="83" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E83" s="2"/>
+      <c r="E83" s="1"/>
     </row>
     <row r="84" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E84" s="2"/>
+      <c r="E84" s="1"/>
     </row>
     <row r="85" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E85" s="2"/>
+      <c r="E85" s="1"/>
     </row>
     <row r="86" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E86" s="2"/>
+      <c r="E86" s="1"/>
     </row>
     <row r="87" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E87" s="2"/>
+      <c r="E87" s="1"/>
     </row>
     <row r="88" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E88" s="2"/>
+      <c r="E88" s="1"/>
     </row>
     <row r="89" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E89" s="2"/>
+      <c r="E89" s="1"/>
     </row>
     <row r="90" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E90" s="2"/>
+      <c r="E90" s="1"/>
     </row>
     <row r="91" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E91" s="2"/>
+      <c r="E91" s="1"/>
     </row>
     <row r="92" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E92" s="2"/>
+      <c r="E92" s="1"/>
     </row>
     <row r="93" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E93" s="2"/>
+      <c r="E93" s="1"/>
     </row>
     <row r="94" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E94" s="2"/>
+      <c r="E94" s="1"/>
     </row>
     <row r="95" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E95" s="2"/>
+      <c r="E95" s="1"/>
     </row>
     <row r="96" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E96" s="2"/>
+      <c r="E96" s="1"/>
     </row>
     <row r="97" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E97" s="2"/>
+      <c r="E97" s="1"/>
     </row>
     <row r="98" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E98" s="2"/>
+      <c r="E98" s="1"/>
     </row>
     <row r="99" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E99" s="2"/>
+      <c r="E99" s="1"/>
     </row>
     <row r="100" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E100" s="2"/>
+      <c r="E100" s="1"/>
     </row>
     <row r="101" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E101" s="2"/>
+      <c r="E101" s="1"/>
     </row>
     <row r="102" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E102" s="2"/>
+      <c r="E102" s="1"/>
     </row>
     <row r="103" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E103" s="2"/>
+      <c r="E103" s="1"/>
     </row>
     <row r="104" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E104" s="2"/>
+      <c r="E104" s="1"/>
     </row>
     <row r="105" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E105" s="2"/>
+      <c r="E105" s="1"/>
     </row>
     <row r="106" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E106" s="2"/>
+      <c r="E106" s="1"/>
     </row>
     <row r="107" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E107" s="2"/>
+      <c r="E107" s="1"/>
     </row>
     <row r="108" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E108" s="2"/>
+      <c r="E108" s="1"/>
     </row>
     <row r="109" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E109" s="2"/>
+      <c r="E109" s="1"/>
     </row>
     <row r="110" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E110" s="2"/>
+      <c r="E110" s="1"/>
     </row>
     <row r="111" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E111" s="2"/>
+      <c r="E111" s="1"/>
     </row>
     <row r="112" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E112" s="2"/>
+      <c r="E112" s="1"/>
     </row>
     <row r="113" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E113" s="2"/>
+      <c r="E113" s="1"/>
     </row>
     <row r="114" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E114" s="2"/>
+      <c r="E114" s="1"/>
     </row>
     <row r="115" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E115" s="2"/>
+      <c r="E115" s="1"/>
     </row>
     <row r="116" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E116" s="2"/>
+      <c r="E116" s="1"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="J11:K12"/>
     <mergeCell ref="Q11:R12"/>
@@ -2159,21 +2153,22 @@
     <mergeCell ref="V6:V7"/>
     <mergeCell ref="J6:N6"/>
     <mergeCell ref="O6:S6"/>
+    <mergeCell ref="Q14:R15"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" showErrorMessage="1" sqref="E6">
+    <dataValidation type="list" showErrorMessage="1" sqref="E6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>Groupes</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation showErrorMessage="1" sqref="F15 C15 C12 S12 L12 F12 L15 C18 K4"/>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="F9 G10:G11">
+    <dataValidation showErrorMessage="1" sqref="K4 F18 C15 C12 S12 L12 F12 F15 C18 L15 S15" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="F9 G10:G11" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" display="www.federation.org"/>
-    <hyperlink ref="A4" r:id="rId2" display="records@federation.org"/>
+    <hyperlink ref="A3" r:id="rId1" display="www.federation.org" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A4" r:id="rId2" display="records@federation.org" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.31527777777777777" right="0.35416666666666669" top="0.39374999999999999" bottom="0.39374999999999999" header="0.51180555555555551" footer="0.51180555555555551"/>
   <pageSetup paperSize="9" scale="72" firstPageNumber="0" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>

</xml_diff>